<commit_message>
feat(dm-pipeline): vidéos publiques + lien dans l'export
- .gitignore : les MP4 dm_videos/*.mp4 ne sont plus ignorés, ils sont
  publiés via GitHub Pages → app.cartefidelavis.com/dm_videos/<slug>-dm.mp4
- dm_videos/jolia-dm.mp4 commité (v9, ~700 KB, 30 s)
- export_demos.py : video_link auto-rempli si MP4 présent, sinon
  status='pending_video' (orange clair dans XLSX) au lieu de 'ready'.
- .github/workflows/gen-dm-videos.yml : workflow manuel (workflow_dispatch)
  qui détecte les restos sans MP4, lance gen_dm_videos.py, régénère les
  coupon-zoom PNG, rafraîchit l'export et commit le tout.
  Secrets requis : HEYGEN_API_KEY, CREATOMATE_API_KEY (à ajouter dans
  Settings → Secrets → Actions du repo).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dm_videos/restaurants_demo.xlsx
+++ b/dm_videos/restaurants_demo.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,11 +40,16 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="0092400E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00166534"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +60,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001A1A1C"/>
         <bgColor rgb="001A1A1C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+        <bgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
@@ -90,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -102,6 +113,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -549,7 +563,7 @@
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>pending_video</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -579,7 +593,7 @@
       <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="4" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>pending_video</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -600,14 +614,18 @@
           <t>https://app.cartefidelavis.com/jolia/demo/</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/dm_videos/jolia-dm.mp4</t>
+        </is>
+      </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Dessert du chef Dessert du chef Dessert</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>ready</t>
         </is>
@@ -639,7 +657,7 @@
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>pending_video</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -669,7 +687,7 @@
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>ready</t>
+          <t>pending_video</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -682,10 +700,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId11"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
anima : visuels de prospection, et validation de la chaine reparee
Chaine complete jouee sur un restaurant qui n'avait encore aucun visuel :
capture HD, mockup iPhone, story et fond video. Quatre etapes sur quatre,
apres la reparation des chemins.

Seule la generation HeyGen reste non testee : la cle n'est pas sur cette
machine, et elle n'a pas a y etre.
</commit_message>
<xml_diff>
--- a/dm_videos/restaurants_demo.xlsx
+++ b/dm_videos/restaurants_demo.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -541,25 +541,21 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>BROTHER SISTER Brunch Lunch Dinner</t>
+          <t>Anima</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/brothersister_paris</t>
+          <t>https://www.instagram.com/anima.paris</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>https://app.cartefidelavis.com/brother-sister-brunch-lunch-dinner/demo/</t>
+          <t>https://app.cartefidelavis.com/anima/demo/</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Boisson chaude offerte</t>
-        </is>
-      </c>
+      <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="4" t="inlineStr">
         <is>
@@ -571,25 +567,21 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Deux Restaurant : Bistrot de chefs</t>
+          <t>Asko</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/deux.ptitdeux</t>
+          <t>https://www.instagram.com/asko.restaurant</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>https://app.cartefidelavis.com/deux-restaurant-bistrot-de-chefs/demo/</t>
+          <t>https://app.cartefidelavis.com/asko/demo/</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Café offert après brunch</t>
-        </is>
-      </c>
+      <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="4" t="inlineStr">
         <is>
@@ -601,33 +593,25 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Jolia</t>
+          <t>Aux Deux Ecus - Brasserie</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/jolia.paris</t>
+          <t>https://www.instagram.com/auxdeuxecus</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>https://app.cartefidelavis.com/jolia/demo/</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>https://app.cartefidelavis.com/dm_videos/jolia-dm.mp4</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Dessert du chef Dessert du chef Dessert</t>
-        </is>
-      </c>
+          <t>https://app.cartefidelavis.com/aux-deux-ecus-brasserie/demo/</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>ready</t>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -635,25 +619,21 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Kafkaf - Paris 11</t>
+          <t>Bacini</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/kafkaf.fr</t>
+          <t>https://www.instagram.com/bacini_pigalle</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>https://app.cartefidelavis.com/kafkaf-paris-11/demo/</t>
+          <t>https://app.cartefidelavis.com/bacini/demo/</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Café offert après brunch</t>
-        </is>
-      </c>
+      <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="4" t="inlineStr">
         <is>
@@ -665,25 +645,21 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Ter.</t>
+          <t>Bistrot Mon café</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>https://www.instagram.com/terparis11</t>
+          <t>https://www.instagram.com/bistrotmoncafe</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>https://app.cartefidelavis.com/ter/demo/</t>
+          <t>https://app.cartefidelavis.com/bistrot-mon-cafe/demo/</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Café offert après brunch</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="4" t="inlineStr">
         <is>
@@ -691,6 +667,712 @@
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>BROTHER SISTER Brunch Lunch Dinner</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/brothersister_paris</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/brother-sister-brunch-lunch-dinner/demo/</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Café Petite</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/cafepetiteparis</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/cafe-petite/demo/</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Casa Loca</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/casa.loca.paris</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/casa-loca/demo/</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>CHOKDEE café</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/chokdeecafe</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/chokdee-cafe/demo/</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Deux Restaurant : Bistrot de chefs</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/deux.ptitdeux</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/deux-restaurant-bistrot-de-chefs/demo/</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Green Deli</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/greendeliparis</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/green-deli/demo/</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>inavoué</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/inavoue_restaurant</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/inavoue/demo/</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>JJ Beaumarchais</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/jjbeaumarchais</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/jj-beaumarchais/demo/</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Jolia</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/jolia.paris</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/jolia/demo/</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/dm_videos/jolia-dm.mp4</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>ready</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Kafkaf - Paris 11</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/kafkaf.fr</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/kafkaf-paris-11/demo/</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>KRAFT</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/kraft.paris</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/kraft/demo/</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Kuisinistan - Restaurant Paris 2</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/kuisinistann</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/kuisinistan-restaurant-paris-2/demo/</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>L'Adada Bar - Bar Paris 14</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/adadabar</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/l-adada-bar-bar-paris-14/demo/</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>L'Atelier du Marché</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/latelierdumarche</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/l-atelier-du-marche/demo/</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>L'atelier Gusto</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lateliergusto</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/l-atelier-gusto/demo/</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Le Bouquet d'Alesia</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lebouquetalesia</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/le-bouquet-d-alesia/demo/</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Le Village Café</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/levillagecafe_paris17</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/le-village-cafe/demo/</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Les Acolytes</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lesacolytes.bistrot</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/les-acolytes/demo/</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Les Mauvais Garçons</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lesmauvaisgarconsparis</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/les-mauvais-garcons/demo/</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Les Ptits Gros</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/les_ptits_gros</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/les-ptits-gros/demo/</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>LIZARD</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/lizardloungeparis</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/lizard/demo/</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Loulou</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/loulou_restaurant</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/loulou/demo/</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>MIURA</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/miura_restaurant_paris</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/miura/demo/</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Princesse</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/princessecafe</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/princesse/demo/</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>T'Cup</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/tcupparis</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/t-cup/demo/</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>Ter.</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/terparis11</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/ter/demo/</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>Terre Restaurant</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/terre.restaurant</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>https://app.cartefidelavis.com/terre-restaurant/demo/</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>pending_video</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -700,11 +1382,65 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId65"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>